<commit_message>
documenting the three appraoches
</commit_message>
<xml_diff>
--- a/docs/modelling_approach.xlsx
+++ b/docs/modelling_approach.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johtorr/Documents/Repos/neural_networks_project_hdm/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7F4CDB-7D8E-8E4A-AED6-4A85D9E4FD8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00DE679-506F-9D46-B0F8-AF7E92F6FBA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="2" xr2:uid="{234F4985-7325-E745-815C-EBE544E9734D}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
     <sheet name="Tabelle3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -413,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -436,20 +436,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1239,33 +1238,33 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="9" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="O9" s="12" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="10" spans="2:19" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="18" t="s">
+      <c r="H10" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="O10" s="16" t="s">
+      <c r="O10" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="P10" s="16"/>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="16"/>
-      <c r="S10" s="16"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="17"/>
+      <c r="S10" s="17"/>
     </row>
     <row r="11" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="O11" s="15"/>
+      <c r="O11" s="14"/>
     </row>
     <row r="12" spans="2:19" ht="17" x14ac:dyDescent="0.25">
       <c r="B12" s="11" t="s">
@@ -1296,20 +1295,18 @@
       <c r="H14" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="O14" s="12"/>
     </row>
     <row r="15" spans="2:19" ht="17" x14ac:dyDescent="0.25">
-      <c r="H15" s="12"/>
       <c r="O15" s="11"/>
     </row>
     <row r="16" spans="2:19" ht="17" x14ac:dyDescent="0.25">
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="H16" s="14" t="s">
+      <c r="H16" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="O16" s="14" t="s">
+      <c r="O16" s="13" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1399,12 +1396,6 @@
       </c>
       <c r="O24" s="11"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="O25" s="12"/>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="H27" s="12"/>
-    </row>
     <row r="28" spans="2:15" ht="17" x14ac:dyDescent="0.25">
       <c r="B28" s="11" t="s">
         <v>33</v>
@@ -1417,13 +1408,13 @@
       </c>
     </row>
     <row r="29" spans="2:15" ht="17" x14ac:dyDescent="0.25">
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="14" t="s">
+      <c r="H29" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="O29" s="14" t="s">
+      <c r="O29" s="13" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed errrors in script
</commit_message>
<xml_diff>
--- a/docs/modelling_approach.xlsx
+++ b/docs/modelling_approach.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johtorr/Documents/Repos/neural_networks_project_hdm/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D9B0E3-2030-424D-9C97-D0F02D64B7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F25AC5E2-27EA-8F44-8B82-DD0563CAAC13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="2" xr2:uid="{234F4985-7325-E745-815C-EBE544E9734D}"/>
   </bookViews>
@@ -1234,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C4425D2-5FFA-4C4B-A495-A22788A789E5}">
-  <dimension ref="B9:S31"/>
+  <dimension ref="B9:S29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="9" spans="2:19" x14ac:dyDescent="0.2">
@@ -1396,41 +1396,41 @@
       </c>
       <c r="O24" s="11"/>
     </row>
+    <row r="26" spans="2:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="B26" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="O26" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="2:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="B27" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="H27" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="O27" s="13" t="s">
+        <v>40</v>
+      </c>
+    </row>
     <row r="28" spans="2:15" ht="17" x14ac:dyDescent="0.25">
       <c r="B28" s="11" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="2:15" ht="17" x14ac:dyDescent="0.25">
-      <c r="B29" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="H29" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="O29" s="13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="30" spans="2:15" ht="17" x14ac:dyDescent="0.25">
-      <c r="B30" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="H30" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="O30" s="11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="31" spans="2:15" ht="17" x14ac:dyDescent="0.25">
-      <c r="O31" s="11"/>
+      <c r="O29" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
added results per model
</commit_message>
<xml_diff>
--- a/docs/modelling_approach.xlsx
+++ b/docs/modelling_approach.xlsx
@@ -8,16 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johtorr/Documents/Repos/neural_networks_project_hdm/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F703579C-52D6-BB44-9625-CD27C9C95A6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75201ABF-048E-4E4D-B265-9E850CC2335A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{234F4985-7325-E745-815C-EBE544E9734D}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="2" xr2:uid="{234F4985-7325-E745-815C-EBE544E9734D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
     <sheet name="Tabelle4" sheetId="4" r:id="rId2"/>
-    <sheet name="Tabelle2" sheetId="2" r:id="rId3"/>
-    <sheet name="Tabelle3" sheetId="3" r:id="rId4"/>
+    <sheet name="Tabelle5" sheetId="5" r:id="rId3"/>
+    <sheet name="Tabelle2" sheetId="2" r:id="rId4"/>
+    <sheet name="Tabelle3" sheetId="3" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tabelle5!$A$1:$I$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="95">
   <si>
     <t>Date</t>
   </si>
@@ -555,6 +559,15 @@
   </si>
   <si>
     <t>Fold</t>
+  </si>
+  <si>
+    <t>Fold2</t>
+  </si>
+  <si>
+    <t>Fold3</t>
+  </si>
+  <si>
+    <t>Average</t>
   </si>
 </sst>
 </file>
@@ -704,10 +717,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1261,7 +1274,7 @@
       <c r="I21" t="s">
         <v>69</v>
       </c>
-      <c r="L21" s="18" t="s">
+      <c r="L21" s="17" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1269,7 +1282,7 @@
       <c r="B22" t="s">
         <v>16</v>
       </c>
-      <c r="L22" s="18" t="s">
+      <c r="L22" s="17" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1283,7 +1296,7 @@
       <c r="D23" t="s">
         <v>64</v>
       </c>
-      <c r="L23" s="18" t="s">
+      <c r="L23" s="17" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1297,7 +1310,7 @@
       <c r="D24" t="s">
         <v>82</v>
       </c>
-      <c r="L24" s="18" t="s">
+      <c r="L24" s="17" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1311,7 +1324,7 @@
       <c r="D25" t="s">
         <v>64</v>
       </c>
-      <c r="L25" s="18" t="s">
+      <c r="L25" s="17" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1325,7 +1338,7 @@
       <c r="D26" t="s">
         <v>82</v>
       </c>
-      <c r="L26" s="18" t="s">
+      <c r="L26" s="17" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1339,7 +1352,7 @@
       <c r="D27" t="s">
         <v>64</v>
       </c>
-      <c r="L27" s="18" t="s">
+      <c r="L27" s="17" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1353,7 +1366,7 @@
       <c r="D28" t="s">
         <v>82</v>
       </c>
-      <c r="L28" s="18" t="s">
+      <c r="L28" s="17" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1380,24 +1393,24 @@
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1468,7 +1481,7 @@
       <c r="D3" t="s">
         <v>65</v>
       </c>
-      <c r="K3" s="18"/>
+      <c r="K3" s="17"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -1483,7 +1496,7 @@
       <c r="D4" t="s">
         <v>65</v>
       </c>
-      <c r="K4" s="18"/>
+      <c r="K4" s="17"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1498,7 +1511,7 @@
       <c r="D5" t="s">
         <v>65</v>
       </c>
-      <c r="K5" s="18"/>
+      <c r="K5" s="17"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -1513,7 +1526,7 @@
       <c r="D6" t="s">
         <v>65</v>
       </c>
-      <c r="K6" s="18"/>
+      <c r="K6" s="17"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1528,7 +1541,7 @@
       <c r="D7" t="s">
         <v>65</v>
       </c>
-      <c r="K7" s="18"/>
+      <c r="K7" s="17"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -1543,7 +1556,7 @@
       <c r="D8" t="s">
         <v>65</v>
       </c>
-      <c r="K8" s="18"/>
+      <c r="K8" s="17"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1558,7 +1571,7 @@
       <c r="D9" t="s">
         <v>65</v>
       </c>
-      <c r="K9" s="18"/>
+      <c r="K9" s="17"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -1573,7 +1586,7 @@
       <c r="D10" t="s">
         <v>65</v>
       </c>
-      <c r="K10" s="18"/>
+      <c r="K10" s="17"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -1900,10 +1913,281 @@
   </sheetData>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A32C5334-F7E7-E34A-95A2-9690A23087D0}">
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" t="s">
+        <v>82</v>
+      </c>
+      <c r="D17" t="s">
+        <v>94</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I1" xr:uid="{A32C5334-F7E7-E34A-95A2-9690A23087D0}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I17">
+      <sortCondition descending="1" ref="B1:B17"/>
+    </sortState>
+  </autoFilter>
+  <phoneticPr fontId="10" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97831699-8ED8-B047-BDB8-038509C9D266}">
   <dimension ref="B9:E28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2103,7 +2387,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C4425D2-5FFA-4C4B-A495-A22788A789E5}">
   <dimension ref="B9:S29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2126,13 +2410,13 @@
       <c r="H10" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="O10" s="17" t="s">
+      <c r="O10" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="P10" s="17"/>
-      <c r="Q10" s="17"/>
-      <c r="R10" s="17"/>
-      <c r="S10" s="17"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="18"/>
+      <c r="S10" s="18"/>
     </row>
     <row r="11" spans="2:19" x14ac:dyDescent="0.2">
       <c r="O11" s="14"/>

</xml_diff>